<commit_message>
Docs: Sydney's latest audit answers (#21–#39)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5675A984-3C9E-FC4A-9FE6-5DF317E4DA76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6B39DA-42D0-AD4E-BACC-6DC92151CE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2008" uniqueCount="500">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2029" uniqueCount="511">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2100,6 +2100,39 @@
   </si>
   <si>
     <t>1. Initials for Monogram in order you want it to appear 2. Name 3. Monogram option 4. Font. 5. Color for monogram (if two toned monogram, add details in additional instructions). 6. Color for Text 7. Color for Border 8. additional instructions 9. name &amp; return address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can we provide a place to upload a photo? If someone wants to provide their own photo, please add $7.50 to the total. Show me what this looks like. We also need to add the cat options. I'll upload the options. Please provide these as an image picker. Or they can choose to updload their own cat photo - if they do, we will remove the background and use the image directly. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can we provide a place to upload a photo? If someone wants to provide their own photo, please add $7.50 to the total. Show me what this looks like. We also need to add the dog options. I'll upload the options. Please provide these as an image picker. Or they can choose to updload their own dog photo - if they do, we will remove the background and use the image directly. </t>
+  </si>
+  <si>
+    <t>Can we provide a place to upload a logo? Regarding placement, we can say that logos will be placed in top center of card unless otherwise requested in additional instructions. In description remove this line: Send us your logo via direct message and we will draft up the card for your revie... can we add a note that if text is added, it will be added to the bottom of the card unless otherwise requested in the additional details section.</t>
+  </si>
+  <si>
+    <t>Let's break out the text into two options. Text for top of card. Names for bottom of card. Remove font option.</t>
+  </si>
+  <si>
+    <t>add: monogram initial for inside wreath 2. monogram color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">let's change text to two options: family name (ex. The Wilson Family), Individual Names (ex. John, Jenny, James, Jerome), remove font option and photo of font options in the photos. </t>
+  </si>
+  <si>
+    <t>remove this from the bottom of the personalization section - Dedications are printed in ~10pt type; leave extra whitespace around content for framing. Remove matching items.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">match prices to other folded notecards. In description, make matching items the shopify listings not etsy. </t>
+  </si>
+  <si>
+    <t>add: monogram style (picker), initials for monogram, name (if no name is desired, type n/a). Update matching items to shopify links</t>
+  </si>
+  <si>
+    <t>Can we provide a place to upload a logo? Regarding placement, we can say that logos will be placed in center of front of card unless otherwise requested in additional instructions.... can we add a note that if text is added, it will be added below the logo on the front of the card unless otherwise requested in the additional details section. make the matching items the shopify links not etsy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add these options. 1. name 2. would you like a monogram in the graduation cap? - if yes, show initials for monogram option 3. do you want thank you in the graduation cap? Yes or no. </t>
   </si>
 </sst>
 </file>
@@ -3022,9 +3055,11 @@
       </c>
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-    </row>
-    <row r="15" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+      <c r="K14" s="7" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -3053,9 +3088,11 @@
         <v>53</v>
       </c>
       <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-    </row>
-    <row r="16" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+      <c r="K15" s="5" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -3084,9 +3121,11 @@
         <v>56</v>
       </c>
       <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-    </row>
-    <row r="17" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+      <c r="K16" s="5" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -3115,7 +3154,9 @@
         <v>56</v>
       </c>
       <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
+      <c r="K17" s="5" t="s">
+        <v>501</v>
+      </c>
     </row>
     <row r="18" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A18" s="7">
@@ -3262,7 +3303,9 @@
         <v>34</v>
       </c>
       <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
+      <c r="K22" s="5" t="s">
+        <v>504</v>
+      </c>
     </row>
     <row r="23" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A23" s="5">
@@ -3293,7 +3336,9 @@
         <v>69</v>
       </c>
       <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
+      <c r="K23" s="5" t="s">
+        <v>505</v>
+      </c>
     </row>
     <row r="24" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A24" s="5">
@@ -3324,7 +3369,9 @@
         <v>72</v>
       </c>
       <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
+      <c r="K24" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="25" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A25" s="5">
@@ -3355,7 +3402,9 @@
         <v>72</v>
       </c>
       <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
+      <c r="K25" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="26" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A26" s="5">
@@ -3386,7 +3435,9 @@
         <v>72</v>
       </c>
       <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
+      <c r="K26" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="27" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A27" s="5">
@@ -3417,7 +3468,9 @@
         <v>72</v>
       </c>
       <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
+      <c r="K27" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="28" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A28" s="5">
@@ -3448,7 +3501,9 @@
         <v>72</v>
       </c>
       <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
+      <c r="K28" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="29" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A29" s="5">
@@ -3479,7 +3534,9 @@
         <v>72</v>
       </c>
       <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
+      <c r="K29" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="30" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A30" s="5">
@@ -3510,7 +3567,9 @@
         <v>72</v>
       </c>
       <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
+      <c r="K30" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="31" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
@@ -3541,7 +3600,9 @@
         <v>72</v>
       </c>
       <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
+      <c r="K31" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="32" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A32" s="5">
@@ -3572,7 +3633,9 @@
         <v>72</v>
       </c>
       <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
+      <c r="K32" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="33" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A33" s="5">
@@ -3603,7 +3666,9 @@
         <v>72</v>
       </c>
       <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
+      <c r="K33" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="34" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A34" s="7">
@@ -3663,7 +3728,9 @@
         <v>72</v>
       </c>
       <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
+      <c r="K35" s="5" t="s">
+        <v>506</v>
+      </c>
     </row>
     <row r="36" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A36" s="5">
@@ -3694,7 +3761,9 @@
         <v>89</v>
       </c>
       <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
+      <c r="K36" s="5" t="s">
+        <v>507</v>
+      </c>
     </row>
     <row r="37" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A37" s="5">
@@ -3725,9 +3794,11 @@
         <v>91</v>
       </c>
       <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-    </row>
-    <row r="38" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+      <c r="K37" s="5" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -3756,7 +3827,9 @@
         <v>53</v>
       </c>
       <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
+      <c r="K38" s="5" t="s">
+        <v>509</v>
+      </c>
     </row>
     <row r="39" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A39" s="7">
@@ -3816,7 +3889,9 @@
         <v>34</v>
       </c>
       <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
+      <c r="K40" s="5" t="s">
+        <v>510</v>
+      </c>
     </row>
     <row r="41" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A41" s="7">

</xml_diff>

<commit_message>
PDP: multi-color questions; review links can preview hidden questions and text label changes
"Colors (pick several)" questions let customers choose more than one color.
Hide-standard-questions and Text-label changes can be staged in draft
fields that only ?drafts=1 links use. Also saves Sydney's latest audit answers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6B39DA-42D0-AD4E-BACC-6DC92151CE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D533A83D-9BD2-0541-99A9-2D6DBBDCCBB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2029" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2035" uniqueCount="517">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2133,6 +2133,27 @@
   </si>
   <si>
     <t xml:space="preserve">add these options. 1. name 2. would you like a monogram in the graduation cap? - if yes, show initials for monogram option 3. do you want thank you in the graduation cap? Yes or no. </t>
+  </si>
+  <si>
+    <t>how can we correct the web address? I don’t know why it doesn’t match. The matching items are not yet created. Let's remove for now. Let's remove copy in the web address as well as long as you can change the web address</t>
+  </si>
+  <si>
+    <t>add monogram option. Replace the monogram option photo with new one. Clean up matching items links.</t>
+  </si>
+  <si>
+    <t>change prices to flat notecards, you can remove the price differential for postcard and cards with envelopes. But still provide the option to choose either postcard and card with envelopes. If they choose postcard, return address will be printed on the back of the card. let's make that clear please.</t>
+  </si>
+  <si>
+    <t>add initials for monogram. Border color. Change text to name. animal option: -Lion
+-Elephant
+-Bunny
+-Giraffe</t>
+  </si>
+  <si>
+    <t>Change text to Name. Remove font. Remove text color. If they choose custom colors, then show a color selecter and allow them to choose multiple colors, put a note that says multiple colors will alternate on the text (add any special instructions in the additional instructions area). remove pdf digital file option and any mention of that in description or title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add sports icon color. </t>
   </si>
 </sst>
 </file>
@@ -4096,7 +4117,9 @@
         <v>110</v>
       </c>
       <c r="J47" s="5"/>
-      <c r="K47" s="5"/>
+      <c r="K47" s="5" t="s">
+        <v>511</v>
+      </c>
     </row>
     <row r="48" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A48" s="7">
@@ -4156,7 +4179,9 @@
         <v>34</v>
       </c>
       <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
+      <c r="K49" s="5" t="s">
+        <v>512</v>
+      </c>
     </row>
     <row r="50" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A50" s="5">
@@ -4187,7 +4212,9 @@
         <v>117</v>
       </c>
       <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
+      <c r="K50" s="5" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="51" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A51" s="7">
@@ -4450,7 +4477,7 @@
       <c r="J59" s="7"/>
       <c r="K59" s="7"/>
     </row>
-    <row r="60" spans="1:11" ht="96" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A60" s="5">
         <v>59</v>
       </c>
@@ -4479,7 +4506,9 @@
         <v>34</v>
       </c>
       <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
+      <c r="K60" s="5" t="s">
+        <v>514</v>
+      </c>
     </row>
     <row r="61" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A61" s="7">
@@ -4655,7 +4684,9 @@
         <v>149</v>
       </c>
       <c r="J66" s="5"/>
-      <c r="K66" s="5"/>
+      <c r="K66" s="5" t="s">
+        <v>515</v>
+      </c>
     </row>
     <row r="67" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A67" s="7">
@@ -4860,7 +4891,9 @@
         <v>53</v>
       </c>
       <c r="J73" s="5"/>
-      <c r="K73" s="5"/>
+      <c r="K73" s="5" t="s">
+        <v>516</v>
+      </c>
     </row>
     <row r="74" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A74" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (#74–#127)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D533A83D-9BD2-0541-99A9-2D6DBBDCCBB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FEB630-307A-6A43-92FE-70F378BB20A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="780" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2035" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="534">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2154,6 +2154,57 @@
   </si>
   <si>
     <t xml:space="preserve">add sports icon color. </t>
+  </si>
+  <si>
+    <t>clean up web address. I don't know why they don't match and remove copy. Clean up matching items links and add the doctor and nurse notepad.</t>
+  </si>
+  <si>
+    <t>prices are ok. Add return address envelope option for $32. in personalization remove font. Change "text" to "name for bottom of card"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clean up web address. Clean up matching items. Update prices to match flat notecard listings. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">clean up matching items. </t>
+  </si>
+  <si>
+    <t>clean up matching items. Remove do not click option.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prices - duplicate other flat notecard sets. Add return address option. </t>
+  </si>
+  <si>
+    <t>clean up matching items line.</t>
+  </si>
+  <si>
+    <t>add itinials for monogram. And change text to name. add monogram color. Clubs color, ball color. Clean up matching items link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">change text to name for top of card. Remove font. Add border color. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">update prices to match other flat notecard prices. Put order with blank envelopes, return envelopes, blank envelopes, etc. </t>
+  </si>
+  <si>
+    <t>update description and remove butteerly. Should say lemon or orange tree. Add option to choose lemon tree or orange tree. Update prices to match. Variant optins should start at 5+blank envelopes, 5+ return, 10+blank, 10+ return. And so on up the ladder. please put in that order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">update web address. Remove the name/address personalization when choosing blank envelope options. Change text to name. remove font option. </t>
+  </si>
+  <si>
+    <t>update prices. Update variant sort order to start with 5 and go up… with blank first then return address. Include matching notepad and artwork link if applicable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">update prices. Remove this text: Preview uses placeholder letters. Final print uses archival ink on cotton paper. </t>
+  </si>
+  <si>
+    <t>update prices. Put blank envelope options before return. So 5+blank, 5+ return, 10+blank, 10+ return, etc.</t>
+  </si>
+  <si>
+    <t>add initials for monogram (2 initials)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add initial for monogram (one initial, if no initial desired, type n/a), choose red bow or blue bow. </t>
   </si>
 </sst>
 </file>
@@ -4953,7 +5004,9 @@
         <v>161</v>
       </c>
       <c r="J75" s="5"/>
-      <c r="K75" s="5"/>
+      <c r="K75" s="5" t="s">
+        <v>517</v>
+      </c>
     </row>
     <row r="76" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A76" s="7">
@@ -5071,7 +5124,9 @@
         <v>169</v>
       </c>
       <c r="J79" s="5"/>
-      <c r="K79" s="5"/>
+      <c r="K79" s="5" t="s">
+        <v>518</v>
+      </c>
     </row>
     <row r="80" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A80" s="7">
@@ -5160,7 +5215,9 @@
         <v>174</v>
       </c>
       <c r="J82" s="5"/>
-      <c r="K82" s="5"/>
+      <c r="K82" s="5" t="s">
+        <v>519</v>
+      </c>
     </row>
     <row r="83" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A83" s="5">
@@ -5191,7 +5248,9 @@
         <v>175</v>
       </c>
       <c r="J83" s="5"/>
-      <c r="K83" s="5"/>
+      <c r="K83" s="5" t="s">
+        <v>520</v>
+      </c>
     </row>
     <row r="84" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A84" s="5">
@@ -5222,7 +5281,9 @@
         <v>179</v>
       </c>
       <c r="J84" s="5"/>
-      <c r="K84" s="5"/>
+      <c r="K84" s="5" t="s">
+        <v>521</v>
+      </c>
     </row>
     <row r="85" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A85" s="7">
@@ -5311,7 +5372,9 @@
         <v>186</v>
       </c>
       <c r="J87" s="5"/>
-      <c r="K87" s="5"/>
+      <c r="K87" s="5" t="s">
+        <v>522</v>
+      </c>
     </row>
     <row r="88" spans="1:11" ht="144" x14ac:dyDescent="0.2">
       <c r="A88" s="7">
@@ -5400,7 +5463,9 @@
         <v>72</v>
       </c>
       <c r="J90" s="5"/>
-      <c r="K90" s="5"/>
+      <c r="K90" s="5" t="s">
+        <v>523</v>
+      </c>
     </row>
     <row r="91" spans="1:11" ht="144" x14ac:dyDescent="0.2">
       <c r="A91" s="7">
@@ -5924,7 +5989,9 @@
         <v>34</v>
       </c>
       <c r="J108" s="5"/>
-      <c r="K108" s="5"/>
+      <c r="K108" s="5" t="s">
+        <v>524</v>
+      </c>
     </row>
     <row r="109" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A109" s="7">
@@ -6129,7 +6196,9 @@
         <v>72</v>
       </c>
       <c r="J115" s="5"/>
-      <c r="K115" s="5"/>
+      <c r="K115" s="5" t="s">
+        <v>525</v>
+      </c>
     </row>
     <row r="116" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A116" s="7">
@@ -6218,7 +6287,9 @@
         <v>242</v>
       </c>
       <c r="J118" s="5"/>
-      <c r="K118" s="5"/>
+      <c r="K118" s="5" t="s">
+        <v>526</v>
+      </c>
     </row>
     <row r="119" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A119" s="5">
@@ -6249,7 +6320,9 @@
         <v>245</v>
       </c>
       <c r="J119" s="5"/>
-      <c r="K119" s="5"/>
+      <c r="K119" s="5" t="s">
+        <v>527</v>
+      </c>
     </row>
     <row r="120" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A120" s="5">
@@ -6280,7 +6353,9 @@
         <v>247</v>
       </c>
       <c r="J120" s="5"/>
-      <c r="K120" s="5"/>
+      <c r="K120" s="5" t="s">
+        <v>528</v>
+      </c>
     </row>
     <row r="121" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A121" s="7">
@@ -6340,7 +6415,9 @@
         <v>242</v>
       </c>
       <c r="J122" s="5"/>
-      <c r="K122" s="5"/>
+      <c r="K122" s="5" t="s">
+        <v>529</v>
+      </c>
     </row>
     <row r="123" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A123" s="7">
@@ -6400,7 +6477,9 @@
         <v>254</v>
       </c>
       <c r="J124" s="5"/>
-      <c r="K124" s="5"/>
+      <c r="K124" s="5" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="125" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A125" s="7">
@@ -6460,7 +6539,9 @@
         <v>242</v>
       </c>
       <c r="J126" s="5"/>
-      <c r="K126" s="5"/>
+      <c r="K126" s="5" t="s">
+        <v>531</v>
+      </c>
     </row>
     <row r="127" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A127" s="5">
@@ -6491,7 +6572,9 @@
         <v>34</v>
       </c>
       <c r="J127" s="5"/>
-      <c r="K127" s="5"/>
+      <c r="K127" s="5" t="s">
+        <v>532</v>
+      </c>
     </row>
     <row r="128" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A128" s="5">
@@ -6522,7 +6605,9 @@
         <v>34</v>
       </c>
       <c r="J128" s="5"/>
-      <c r="K128" s="5"/>
+      <c r="K128" s="5" t="s">
+        <v>533</v>
+      </c>
     </row>
     <row r="129" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A129" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (#131–#135)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FEB630-307A-6A43-92FE-70F378BB20A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AC7BEB-051B-924F-B6FE-95DB707DF103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="780" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="538">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2198,6 +2198,9 @@
     <t xml:space="preserve">update prices. Remove this text: Preview uses placeholder letters. Final print uses archival ink on cotton paper. </t>
   </si>
   <si>
+    <t xml:space="preserve">update prices. </t>
+  </si>
+  <si>
     <t>update prices. Put blank envelope options before return. So 5+blank, 5+ return, 10+blank, 10+ return, etc.</t>
   </si>
   <si>
@@ -2205,6 +2208,15 @@
   </si>
   <si>
     <t xml:space="preserve">add initial for monogram (one initial, if no initial desired, type n/a), choose red bow or blue bow. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">name &amp; return address should not be showing on blank envelopes. Add matching item links (also include doctor items as well as nurse). in personalization change "text" to name. I don't want them to think the RN by the icon is going to be in a different font, the intent is for that font to stay the same as what they see on the product examples but they can change the font of the name. if you can think of any good ways to make that clear, let me know. </t>
+  </si>
+  <si>
+    <t>update prices. Order variations to go blank, then return address, then blank, then return address, etc.</t>
+  </si>
+  <si>
+    <t>update prices</t>
   </si>
 </sst>
 </file>
@@ -6540,7 +6552,7 @@
       </c>
       <c r="J126" s="5"/>
       <c r="K126" s="5" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="96" x14ac:dyDescent="0.2">
@@ -6573,7 +6585,7 @@
       </c>
       <c r="J127" s="5"/>
       <c r="K127" s="5" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="96" x14ac:dyDescent="0.2">
@@ -6606,7 +6618,7 @@
       </c>
       <c r="J128" s="5"/>
       <c r="K128" s="5" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="96" x14ac:dyDescent="0.2">
@@ -6696,7 +6708,7 @@
       <c r="J131" s="7"/>
       <c r="K131" s="7"/>
     </row>
-    <row r="132" spans="1:11" ht="112" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A132" s="5">
         <v>131</v>
       </c>
@@ -6725,7 +6737,9 @@
         <v>34</v>
       </c>
       <c r="J132" s="5"/>
-      <c r="K132" s="5"/>
+      <c r="K132" s="5" t="s">
+        <v>535</v>
+      </c>
     </row>
     <row r="133" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A133" s="5">
@@ -6756,7 +6770,9 @@
         <v>267</v>
       </c>
       <c r="J133" s="5"/>
-      <c r="K133" s="5"/>
+      <c r="K133" s="5" t="s">
+        <v>536</v>
+      </c>
     </row>
     <row r="134" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A134" s="5">
@@ -6787,7 +6803,9 @@
         <v>242</v>
       </c>
       <c r="J134" s="5"/>
-      <c r="K134" s="5"/>
+      <c r="K134" s="5" t="s">
+        <v>531</v>
+      </c>
     </row>
     <row r="135" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A135" s="7">
@@ -6847,7 +6865,9 @@
         <v>242</v>
       </c>
       <c r="J136" s="5"/>
-      <c r="K136" s="5"/>
+      <c r="K136" s="5" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="137" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A137" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (#138–#145)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AC7BEB-051B-924F-B6FE-95DB707DF103}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F8590F-E53F-034A-A9DC-66006CE6CCDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="780" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2061" uniqueCount="543">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2217,6 +2217,21 @@
   </si>
   <si>
     <t>update prices</t>
+  </si>
+  <si>
+    <t>add pinapple placement - top center or bottom left.</t>
+  </si>
+  <si>
+    <t>clean up matching items links</t>
+  </si>
+  <si>
+    <t>update prices. Include matching items list (include the barrell cactus too)</t>
+  </si>
+  <si>
+    <t>include matching items links</t>
+  </si>
+  <si>
+    <t>make sure photos wrap around so they are not justting into the personalization section.</t>
   </si>
 </sst>
 </file>
@@ -6956,7 +6971,9 @@
         <v>278</v>
       </c>
       <c r="J139" s="5"/>
-      <c r="K139" s="5"/>
+      <c r="K139" s="5" t="s">
+        <v>538</v>
+      </c>
     </row>
     <row r="140" spans="1:11" ht="144" x14ac:dyDescent="0.2">
       <c r="A140" s="5">
@@ -6987,7 +7004,9 @@
         <v>72</v>
       </c>
       <c r="J140" s="5"/>
-      <c r="K140" s="5"/>
+      <c r="K140" s="5" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="141" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A141" s="7">
@@ -7076,7 +7095,9 @@
         <v>242</v>
       </c>
       <c r="J143" s="5"/>
-      <c r="K143" s="5"/>
+      <c r="K143" s="5" t="s">
+        <v>540</v>
+      </c>
     </row>
     <row r="144" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A144" s="7">
@@ -7136,7 +7157,9 @@
         <v>287</v>
       </c>
       <c r="J145" s="5"/>
-      <c r="K145" s="5"/>
+      <c r="K145" s="5" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="146" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A146" s="5">
@@ -7167,7 +7190,9 @@
         <v>290</v>
       </c>
       <c r="J146" s="5"/>
-      <c r="K146" s="5"/>
+      <c r="K146" s="5" t="s">
+        <v>542</v>
+      </c>
     </row>
     <row r="147" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A147" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (#149–#168)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F8590F-E53F-034A-A9DC-66006CE6CCDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58EA67DE-CB85-964A-8D8C-FAE459FE63D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20" yWindow="780" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2061" uniqueCount="543">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2073" uniqueCount="555">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2232,6 +2232,42 @@
   </si>
   <si>
     <t>make sure photos wrap around so they are not justting into the personalization section.</t>
+  </si>
+  <si>
+    <t>clean up matchign items</t>
+  </si>
+  <si>
+    <t>this product should not be active. Please move to draft.</t>
+  </si>
+  <si>
+    <t>update prices. Put variables in correct order.</t>
+  </si>
+  <si>
+    <t>clean up matching items</t>
+  </si>
+  <si>
+    <t>update prices. Wrap photos around so they are not jutting into personalization section</t>
+  </si>
+  <si>
+    <t>break out text to "camp name" and "name for bottom of card". Remove font. For color, change it to "color" and make a note that says text and icons will be in this color. Clean up matching items link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">update prices. Arrange variables in correct order i.e. blank then return address. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">include matching item links for all tennis items. </t>
+  </si>
+  <si>
+    <t>add track &amp; field icon color</t>
+  </si>
+  <si>
+    <t>add air force icon option - can you get the icons from the images? There are two options. Add matchign items in description</t>
+  </si>
+  <si>
+    <t>add matchign items links. Add us army icon option - 1) logo 2) symbol 3) rank insignia. If they choose 3, another option should appear that allows them to type in their rank insignia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">update prices. Remove icon color. Clean up matching item links. </t>
   </si>
 </sst>
 </file>
@@ -7310,7 +7346,9 @@
         <v>72</v>
       </c>
       <c r="J150" s="5"/>
-      <c r="K150" s="5"/>
+      <c r="K150" s="5" t="s">
+        <v>543</v>
+      </c>
     </row>
     <row r="151" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A151" s="5">
@@ -7341,7 +7379,9 @@
         <v>300</v>
       </c>
       <c r="J151" s="5"/>
-      <c r="K151" s="5"/>
+      <c r="K151" s="5" t="s">
+        <v>544</v>
+      </c>
     </row>
     <row r="152" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A152" s="5">
@@ -7372,7 +7412,9 @@
         <v>242</v>
       </c>
       <c r="J152" s="5"/>
-      <c r="K152" s="5"/>
+      <c r="K152" s="5" t="s">
+        <v>545</v>
+      </c>
     </row>
     <row r="153" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A153" s="5">
@@ -7403,7 +7445,9 @@
         <v>72</v>
       </c>
       <c r="J153" s="5"/>
-      <c r="K153" s="5"/>
+      <c r="K153" s="5" t="s">
+        <v>546</v>
+      </c>
     </row>
     <row r="154" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A154" s="5">
@@ -7434,7 +7478,9 @@
         <v>242</v>
       </c>
       <c r="J154" s="5"/>
-      <c r="K154" s="5"/>
+      <c r="K154" s="5" t="s">
+        <v>547</v>
+      </c>
     </row>
     <row r="155" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A155" s="5">
@@ -7465,7 +7511,9 @@
         <v>34</v>
       </c>
       <c r="J155" s="5"/>
-      <c r="K155" s="5"/>
+      <c r="K155" s="5" t="s">
+        <v>548</v>
+      </c>
     </row>
     <row r="156" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A156" s="5">
@@ -7496,7 +7544,9 @@
         <v>242</v>
       </c>
       <c r="J156" s="5"/>
-      <c r="K156" s="5"/>
+      <c r="K156" s="5" t="s">
+        <v>549</v>
+      </c>
     </row>
     <row r="157" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A157" s="7">
@@ -7585,7 +7635,9 @@
         <v>315</v>
       </c>
       <c r="J159" s="5"/>
-      <c r="K159" s="5"/>
+      <c r="K159" s="5" t="s">
+        <v>550</v>
+      </c>
     </row>
     <row r="160" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A160" s="7">
@@ -7674,7 +7726,9 @@
         <v>53</v>
       </c>
       <c r="J162" s="5"/>
-      <c r="K162" s="5"/>
+      <c r="K162" s="5" t="s">
+        <v>551</v>
+      </c>
     </row>
     <row r="163" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A163" s="5">
@@ -7705,7 +7759,9 @@
         <v>321</v>
       </c>
       <c r="J163" s="5"/>
-      <c r="K163" s="5"/>
+      <c r="K163" s="5" t="s">
+        <v>552</v>
+      </c>
     </row>
     <row r="164" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A164" s="5">
@@ -7736,7 +7792,9 @@
         <v>72</v>
       </c>
       <c r="J164" s="5"/>
-      <c r="K164" s="5"/>
+      <c r="K164" s="5" t="s">
+        <v>553</v>
+      </c>
     </row>
     <row r="165" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A165" s="7">
@@ -7883,7 +7941,9 @@
         <v>89</v>
       </c>
       <c r="J169" s="5"/>
-      <c r="K169" s="5"/>
+      <c r="K169" s="5" t="s">
+        <v>554</v>
+      </c>
     </row>
     <row r="170" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A170" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (#171–#180, notepads #1–#3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58EA67DE-CB85-964A-8D8C-FAE459FE63D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AFEBE6D-5D42-3641-9C3C-F001D1E27871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="780" windowWidth="34560" windowHeight="20340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2073" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2079" uniqueCount="560">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2268,6 +2268,21 @@
   </si>
   <si>
     <t xml:space="preserve">update prices. Remove icon color. Clean up matching item links. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">change the personalization like you did for the encouraging bible verse pack where there is an envelope option of eithe r blank envelopes at $25 or return address at $32. </t>
+  </si>
+  <si>
+    <t>add envelope option. Blank envelopes at $22.00 or return address printed on envelopes at $30.00. remove the rest of the personalization other than name/return address for return address envelopes.</t>
+  </si>
+  <si>
+    <t>remove do not click option</t>
+  </si>
+  <si>
+    <t>update variants to the same as the notepads with the same szies and prices. Change text to "name", remove font</t>
+  </si>
+  <si>
+    <t>text should be initials for monogram in order you want it to appear. Remove font. Copy color options from the block monogram notecards. Add matching product link.</t>
   </si>
 </sst>
 </file>
@@ -8032,7 +8047,9 @@
         <v>338</v>
       </c>
       <c r="J172" s="5"/>
-      <c r="K172" s="5"/>
+      <c r="K172" s="5" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="173" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A173" s="7">
@@ -8150,7 +8167,9 @@
         <v>346</v>
       </c>
       <c r="J176" s="5"/>
-      <c r="K176" s="5"/>
+      <c r="K176" s="5" t="s">
+        <v>555</v>
+      </c>
     </row>
     <row r="177" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A177" s="7">
@@ -8297,7 +8316,9 @@
         <v>356</v>
       </c>
       <c r="J181" s="5"/>
-      <c r="K181" s="5"/>
+      <c r="K181" s="5" t="s">
+        <v>556</v>
+      </c>
     </row>
     <row r="182" spans="1:11" ht="128" x14ac:dyDescent="0.2">
       <c r="A182" s="7">
@@ -8964,7 +8985,9 @@
         <v>321</v>
       </c>
       <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
+      <c r="K2" s="5" t="s">
+        <v>557</v>
+      </c>
     </row>
     <row r="3" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A3" s="5">
@@ -8995,7 +9018,9 @@
         <v>363</v>
       </c>
       <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
+      <c r="K3" s="5" t="s">
+        <v>558</v>
+      </c>
     </row>
     <row r="4" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A4" s="5">
@@ -9026,7 +9051,9 @@
         <v>34</v>
       </c>
       <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
+      <c r="K4" s="5" t="s">
+        <v>559</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A5" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (notepads #5–#8)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AFEBE6D-5D42-3641-9C3C-F001D1E27871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F84DFC73-11CD-CC48-894B-609F5DAB2512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2079" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="563">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2283,6 +2283,17 @@
   </si>
   <si>
     <t>text should be initials for monogram in order you want it to appear. Remove font. Copy color options from the block monogram notecards. Add matching product link.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">let's copy the format the of the business logo notecards for the personalization options. </t>
+  </si>
+  <si>
+    <t>replace text with name. remove this from description: Common Text Ideas
+"I'd Rather Be Duck Hunting"
+"Things To Do After Duck Hunting"</t>
+  </si>
+  <si>
+    <t>monogram initials (2 initials). In description add that this is a2 letter monogram and that the last name initial will be in the back and the front name initial will be in the front of the monogram. Add monogram border color + monogram fill color. Change text to "name"</t>
   </si>
 </sst>
 </file>
@@ -9113,7 +9124,9 @@
         <v>53</v>
       </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
+      <c r="K6" s="5" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="112" x14ac:dyDescent="0.2">
       <c r="A7" s="7">
@@ -9173,9 +9186,11 @@
         <v>53</v>
       </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-    </row>
-    <row r="9" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+      <c r="K8" s="5" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -9204,7 +9219,9 @@
         <v>34</v>
       </c>
       <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
+      <c r="K9" s="5" t="s">
+        <v>562</v>
+      </c>
     </row>
     <row r="10" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A10" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (notepads #10–#17)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F84DFC73-11CD-CC48-894B-609F5DAB2512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EFF80EE-9F74-B141-9DF4-9E0E3309BD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2088" uniqueCount="569">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2294,6 +2294,26 @@
   </si>
   <si>
     <t>monogram initials (2 initials). In description add that this is a2 letter monogram and that the last name initial will be in the back and the front name initial will be in the front of the monogram. Add monogram border color + monogram fill color. Change text to "name"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">copy personalization option for the fall wreath notecards. Update matching items. </t>
+  </si>
+  <si>
+    <t>remove this from the descripton - Common Text Ideas
+"I'd Rather Be Playing Fishing"
+"Things To Do After Catching Trout"</t>
+  </si>
+  <si>
+    <t>copy personalization options from the holiiay wreath and bow notecards. Include matching items links</t>
+  </si>
+  <si>
+    <t>include matching item links</t>
+  </si>
+  <si>
+    <t>hmm. Yes one of these lotus notepads looks like a dupe. Pleaes deactivate one but I want to make sure it's not the one connected with etsy/faire</t>
+  </si>
+  <si>
+    <t>include a saying option in personalization 1) I'd Rather Be Playing Mahjong 2) Things To Do After Mahjong 3) Custom - if 3 is selected, open up a text box for them to put their saying 4)none. Change "Text" to "name". Include matching items links</t>
   </si>
 </sst>
 </file>
@@ -9281,7 +9301,9 @@
         <v>376</v>
       </c>
       <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
+      <c r="K11" s="5" t="s">
+        <v>563</v>
+      </c>
     </row>
     <row r="12" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A12" s="5">
@@ -9312,7 +9334,9 @@
         <v>53</v>
       </c>
       <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
+      <c r="K12" s="5" t="s">
+        <v>564</v>
+      </c>
     </row>
     <row r="13" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A13" s="7">
@@ -9372,7 +9396,9 @@
         <v>34</v>
       </c>
       <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
+      <c r="K14" s="5" t="s">
+        <v>565</v>
+      </c>
     </row>
     <row r="15" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A15" s="7">
@@ -9432,7 +9458,9 @@
         <v>385</v>
       </c>
       <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
+      <c r="K16" s="5" t="s">
+        <v>566</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
@@ -9463,9 +9491,11 @@
         <v>387</v>
       </c>
       <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-    </row>
-    <row r="18" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+      <c r="K17" s="5" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -9494,7 +9524,9 @@
         <v>53</v>
       </c>
       <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
+      <c r="K18" s="5" t="s">
+        <v>568</v>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A19" s="5">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (notepads #18, #23, #28)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EFF80EE-9F74-B141-9DF4-9E0E3309BD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35392FF-309B-1444-AF9B-01C05E9BE9FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2088" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2091" uniqueCount="572">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2314,6 +2314,15 @@
   </si>
   <si>
     <t>include a saying option in personalization 1) I'd Rather Be Playing Mahjong 2) Things To Do After Mahjong 3) Custom - if 3 is selected, open up a text box for them to put their saying 4)none. Change "Text" to "name". Include matching items links</t>
+  </si>
+  <si>
+    <t>add intials for monogram (2 initials) include a saying option in personalization 1) I'd Rather Be Playing Mahjong 2) Things To Do After Mahjong 3) Custom - if 3 is selected, open up a text box for them to put their saying 4)none. Change "Text" to "name". Include matching items links</t>
+  </si>
+  <si>
+    <t>clean up matching item links. add the cat images as options. Add option to upload cat photo like the cat notecards. In description remove the mention of "don't see us your breed, let us know" and replace with choose from our library of breed images or proivde an image of your cat. Ok quesiton, if they want to add more than one cat, how do we handle that? give me your ideas. i'd also like to charge extra for more than one cat... maybe like $2.50 for each additional cat. waht do you think?</t>
+  </si>
+  <si>
+    <t>add matching items link (include nurse items). Add icon color. Remove details and text under the personalization section.</t>
   </si>
 </sst>
 </file>
@@ -9528,7 +9537,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -9557,7 +9566,9 @@
         <v>34</v>
       </c>
       <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
+      <c r="K19" s="5" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="20" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A20" s="7">
@@ -9675,7 +9686,7 @@
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
     </row>
-    <row r="24" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" ht="144" x14ac:dyDescent="0.2">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -9704,7 +9715,9 @@
         <v>397</v>
       </c>
       <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
+      <c r="K24" s="5" t="s">
+        <v>570</v>
+      </c>
     </row>
     <row r="25" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A25" s="7">
@@ -9851,7 +9864,9 @@
         <v>321</v>
       </c>
       <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
+      <c r="K29" s="5" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="30" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A30" s="5">

</xml_diff>

<commit_message>
PDP: stationery gift sets ask notecard questions, not gift-tag ones
The Hydrangea and Lotus gift sets mention "Enclosure Cards" in their titles,
so they were treated as gift tags and their Text box said "Appears under
'a gift from' on the tag." Also saves Sydney's latest audit answers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35392FF-309B-1444-AF9B-01C05E9BE9FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A7626E-A2D1-3A48-A2E0-34762FA2EF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="900" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2091" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2095" uniqueCount="576">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2323,6 +2323,18 @@
   </si>
   <si>
     <t>add matching items link (include nurse items). Add icon color. Remove details and text under the personalization section.</t>
+  </si>
+  <si>
+    <t>update with dog option images and copy the cat notepad personalization. Clean up matching items links</t>
+  </si>
+  <si>
+    <t xml:space="preserve">initials for monogram, up to 3 allowed. </t>
+  </si>
+  <si>
+    <t>name for bottom of notepad. Intiiasl for monogram (up to 3 initials, last name will go on bottom), saying for top of notepad: I'd rather be playing golf, things to do after golf, custom (if custom, open up a text box), or none. Color for monogram. Color for golf icons. clean up matching items list.</t>
+  </si>
+  <si>
+    <t>under text it says "Appears under "a gift from" on the tag." - remove that. On description change to: "Customize name, colors &amp; font for text"</t>
   </si>
 </sst>
 </file>
@@ -8956,7 +8968,8 @@
     <col min="4" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="38" customWidth="1"/>
-    <col min="8" max="9" width="52" customWidth="1"/>
+    <col min="8" max="8" width="36.33203125" customWidth="1"/>
+    <col min="9" max="9" width="45.6640625" customWidth="1"/>
     <col min="10" max="10" width="7" customWidth="1"/>
     <col min="11" max="11" width="48" customWidth="1"/>
   </cols>
@@ -9897,7 +9910,9 @@
         <v>56</v>
       </c>
       <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
+      <c r="K30" s="5" t="s">
+        <v>572</v>
+      </c>
     </row>
     <row r="31" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A31" s="5">
@@ -9928,7 +9943,9 @@
         <v>34</v>
       </c>
       <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
+      <c r="K31" s="5" t="s">
+        <v>573</v>
+      </c>
     </row>
     <row r="32" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A32" s="7">
@@ -9959,7 +9976,7 @@
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
     </row>
-    <row r="33" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -9988,7 +10005,9 @@
         <v>91</v>
       </c>
       <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
+      <c r="K33" s="5" t="s">
+        <v>574</v>
+      </c>
     </row>
     <row r="34" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A34" s="7">
@@ -10077,7 +10096,9 @@
         <v>414</v>
       </c>
       <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
+      <c r="K36" s="5" t="s">
+        <v>575</v>
+      </c>
     </row>
     <row r="37" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A37" s="7">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (notepads #36–#43)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A7626E-A2D1-3A48-A2E0-34762FA2EF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8588072A-A9C4-3C48-A28B-255E1DCB9239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="900" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="How to use" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2095" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="583">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2335,6 +2335,27 @@
   </si>
   <si>
     <t>under text it says "Appears under "a gift from" on the tag." - remove that. On description change to: "Customize name, colors &amp; font for text"</t>
+  </si>
+  <si>
+    <t>1. Name 2. additional instructions - remove everything else</t>
+  </si>
+  <si>
+    <t>name for bottom of notepad.  saying for top of notepad: I'd rather be playing lacrosse, things to do after lacrosse, custom (if custom, open up a text box), or none. Color for sticks. Color for ball. clean up matching items list.</t>
+  </si>
+  <si>
+    <t>clean up web address.</t>
+  </si>
+  <si>
+    <t>remove customize border color in the description. We will not be offering an option for border color.</t>
+  </si>
+  <si>
+    <t>clean up variants &amp; prices, should be the same as other notepad sizes. Increase size of text box, should have room for 150 characters. Take marine corps image options and put them as a image picker like the air force/army products. Put matching item links.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">match personalization structure of monogram notecards. Clean up matching item links. </t>
+  </si>
+  <si>
+    <t>match personalization structure of Personalized Fall Plaid Notepad with Monogram. Include matching items links for the blue/navy tartan plaid</t>
   </si>
 </sst>
 </file>
@@ -10127,7 +10148,9 @@
       </c>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
+      <c r="K37" s="7" t="s">
+        <v>576</v>
+      </c>
     </row>
     <row r="38" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A38" s="5">
@@ -10158,7 +10181,9 @@
         <v>72</v>
       </c>
       <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
+      <c r="K38" s="5" t="s">
+        <v>577</v>
+      </c>
     </row>
     <row r="39" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A39" s="5">
@@ -10189,7 +10214,9 @@
         <v>418</v>
       </c>
       <c r="J39" s="5"/>
-      <c r="K39" s="5"/>
+      <c r="K39" s="5" t="s">
+        <v>578</v>
+      </c>
     </row>
     <row r="40" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A40" s="5">
@@ -10220,7 +10247,9 @@
         <v>414</v>
       </c>
       <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
+      <c r="K40" s="5" t="s">
+        <v>579</v>
+      </c>
     </row>
     <row r="41" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A41" s="7">
@@ -10251,7 +10280,7 @@
       <c r="J41" s="7"/>
       <c r="K41" s="7"/>
     </row>
-    <row r="42" spans="1:11" ht="64" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" ht="80" x14ac:dyDescent="0.2">
       <c r="A42" s="5">
         <v>41</v>
       </c>
@@ -10280,7 +10309,9 @@
         <v>424</v>
       </c>
       <c r="J42" s="5"/>
-      <c r="K42" s="5"/>
+      <c r="K42" s="5" t="s">
+        <v>580</v>
+      </c>
     </row>
     <row r="43" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A43" s="5">
@@ -10311,7 +10342,9 @@
         <v>34</v>
       </c>
       <c r="J43" s="5"/>
-      <c r="K43" s="5"/>
+      <c r="K43" s="5" t="s">
+        <v>581</v>
+      </c>
     </row>
     <row r="44" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A44" s="5">
@@ -10342,7 +10375,9 @@
         <v>34</v>
       </c>
       <c r="J44" s="5"/>
-      <c r="K44" s="5"/>
+      <c r="K44" s="5" t="s">
+        <v>582</v>
+      </c>
     </row>
     <row r="45" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A45" s="7">
@@ -10822,7 +10857,7 @@
       <c r="J60" s="5"/>
       <c r="K60" s="5"/>
     </row>
-    <row r="61" spans="1:11" ht="80" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A61" s="5">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (notepads #48–#57)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8588072A-A9C4-3C48-A28B-255E1DCB9239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558E5EE6-53AA-BA4E-897D-0A4D6E9C0650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2107" uniqueCount="588">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2356,6 +2356,21 @@
   </si>
   <si>
     <t>match personalization structure of Personalized Fall Plaid Notepad with Monogram. Include matching items links for the blue/navy tartan plaid</t>
+  </si>
+  <si>
+    <t>copy personalization from the polo monogram notecards. Clean up matching item links.</t>
+  </si>
+  <si>
+    <t>change text to name. remove all other perosnlization other than "additional requests"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">remove first two photos. Change open text field to 150 characters. add ski color option: red or pink skis. Add matching item link. </t>
+  </si>
+  <si>
+    <t>add border color combo: Pink color combo, green color combo. Add links  to any other skiing products</t>
+  </si>
+  <si>
+    <t>clean up matching items. Personalization. Add saying for top of notepad: "I'd rather be playing soccer", "things to do after soccer", custom, or none. Change text to name for bottom of notepad</t>
   </si>
 </sst>
 </file>
@@ -10524,7 +10539,9 @@
         <v>376</v>
       </c>
       <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
+      <c r="K49" s="5" t="s">
+        <v>583</v>
+      </c>
     </row>
     <row r="50" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A50" s="7">
@@ -10584,7 +10601,9 @@
         <v>435</v>
       </c>
       <c r="J51" s="5"/>
-      <c r="K51" s="5"/>
+      <c r="K51" s="5" t="s">
+        <v>584</v>
+      </c>
     </row>
     <row r="52" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A52" s="7">
@@ -10702,7 +10721,9 @@
         <v>440</v>
       </c>
       <c r="J55" s="5"/>
-      <c r="K55" s="5"/>
+      <c r="K55" s="5" t="s">
+        <v>585</v>
+      </c>
     </row>
     <row r="56" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A56" s="5">
@@ -10733,7 +10754,9 @@
         <v>442</v>
       </c>
       <c r="J56" s="5"/>
-      <c r="K56" s="5"/>
+      <c r="K56" s="5" t="s">
+        <v>586</v>
+      </c>
     </row>
     <row r="57" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A57" s="7">
@@ -10793,7 +10816,9 @@
         <v>72</v>
       </c>
       <c r="J58" s="5"/>
-      <c r="K58" s="5"/>
+      <c r="K58" s="5" t="s">
+        <v>587</v>
+      </c>
     </row>
     <row r="59" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A59" s="5">

</xml_diff>

<commit_message>
Docs: Sydney's latest audit answers (notepads #58–#75)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KFkzRMKTGvAFZoGGUJ76Y9
</commit_message>
<xml_diff>
--- a/docs/Product-Audit-Notecards-Notepads.xlsx
+++ b/docs/Product-Audit-Notecards-Notepads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sydneywilson/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{558E5EE6-53AA-BA4E-897D-0A4D6E9C0650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E69B95-88C7-A54A-9812-2F9C544B17E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20340" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2107" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2119" uniqueCount="599">
   <si>
     <t>Product audit — Notecards &amp; Notepads</t>
   </si>
@@ -2371,6 +2371,39 @@
   </si>
   <si>
     <t>clean up matching items. Personalization. Add saying for top of notepad: "I'd rather be playing soccer", "things to do after soccer", custom, or none. Change text to name for bottom of notepad</t>
+  </si>
+  <si>
+    <t>match personalization from the camp notecards. Clean up matching items links.</t>
+  </si>
+  <si>
+    <t>match personalization from the navy/blue tartan notepad. But the name text should just say "name" because it will go on the top of the notepad for this one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">match web address. Matching tiems include any teacher specific prodcuts. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">in description, put default text will say "from the desk of" unless otherwise requested. Add border color. Remove font include maching item links for any teacher products. </t>
+  </si>
+  <si>
+    <t>put product in draft</t>
+  </si>
+  <si>
+    <t>clean up web address. Clean up matching item links. Copy personalization options from air force notecards.</t>
+  </si>
+  <si>
+    <t>in description add "border colors will be as-shown" . You can customize font/color for text</t>
+  </si>
+  <si>
+    <t>put into draft</t>
+  </si>
+  <si>
+    <t>copy soccer notepad personalization options but put water polo into the saying options. Clean up matching items link.</t>
+  </si>
+  <si>
+    <t>clean up matching items link. Copy personalization format for marine corps notepad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">make the flowers an image picker. </t>
   </si>
 </sst>
 </file>
@@ -10849,7 +10882,9 @@
         <v>34</v>
       </c>
       <c r="J59" s="5"/>
-      <c r="K59" s="5"/>
+      <c r="K59" s="5" t="s">
+        <v>588</v>
+      </c>
     </row>
     <row r="60" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A60" s="5">
@@ -10880,7 +10915,9 @@
         <v>34</v>
       </c>
       <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
+      <c r="K60" s="5" t="s">
+        <v>589</v>
+      </c>
     </row>
     <row r="61" spans="1:11" ht="96" x14ac:dyDescent="0.2">
       <c r="A61" s="5">
@@ -10911,7 +10948,9 @@
         <v>449</v>
       </c>
       <c r="J61" s="5"/>
-      <c r="K61" s="5"/>
+      <c r="K61" s="5" t="s">
+        <v>590</v>
+      </c>
     </row>
     <row r="62" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A62" s="5">
@@ -10942,7 +10981,9 @@
         <v>72</v>
       </c>
       <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
+      <c r="K62" s="5" t="s">
+        <v>591</v>
+      </c>
     </row>
     <row r="63" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A63" s="7">
@@ -11002,7 +11043,9 @@
         <v>424</v>
       </c>
       <c r="J64" s="5"/>
-      <c r="K64" s="5"/>
+      <c r="K64" s="5" t="s">
+        <v>592</v>
+      </c>
     </row>
     <row r="65" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A65" s="5">
@@ -11033,7 +11076,9 @@
         <v>455</v>
       </c>
       <c r="J65" s="5"/>
-      <c r="K65" s="5"/>
+      <c r="K65" s="5" t="s">
+        <v>593</v>
+      </c>
     </row>
     <row r="66" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A66" s="7">
@@ -11093,7 +11138,9 @@
         <v>459</v>
       </c>
       <c r="J67" s="5"/>
-      <c r="K67" s="5"/>
+      <c r="K67" s="5" t="s">
+        <v>594</v>
+      </c>
     </row>
     <row r="68" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A68" s="5">
@@ -11124,7 +11171,9 @@
         <v>461</v>
       </c>
       <c r="J68" s="5"/>
-      <c r="K68" s="5"/>
+      <c r="K68" s="5" t="s">
+        <v>595</v>
+      </c>
     </row>
     <row r="69" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A69" s="7">
@@ -11184,7 +11233,9 @@
         <v>34</v>
       </c>
       <c r="J70" s="5"/>
-      <c r="K70" s="5"/>
+      <c r="K70" s="5" t="s">
+        <v>596</v>
+      </c>
     </row>
     <row r="71" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A71" s="5">
@@ -11215,7 +11266,9 @@
         <v>53</v>
       </c>
       <c r="J71" s="5"/>
-      <c r="K71" s="5"/>
+      <c r="K71" s="5" t="s">
+        <v>539</v>
+      </c>
     </row>
     <row r="72" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A72" s="7">
@@ -11304,7 +11357,9 @@
         <v>72</v>
       </c>
       <c r="J74" s="5"/>
-      <c r="K74" s="5"/>
+      <c r="K74" s="5" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="75" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A75" s="7">
@@ -11364,7 +11419,9 @@
         <v>56</v>
       </c>
       <c r="J76" s="5"/>
-      <c r="K76" s="5"/>
+      <c r="K76" s="5" t="s">
+        <v>598</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K76" xr:uid="{00000000-0009-0000-0000-000002000000}"/>

</xml_diff>